<commit_message>
docs: v0 development freeze (5-Sep) + mentor workbooks refreshed to 169-row state
- spec.md: §7 items 15-19 (both real rounds, the two KPI-exclusion incidents,
  the recalibration policy + tt_ob_lb flag) and §9 freeze record.
- reports/: PROVEN_6_Trust_Report + UQ_Prediction_Report re-fit to current
  per-KPI row counts; README.md documents the recalibration check.
  UQ_Method_Benchmark deliberately NOT re-run (mentor-approved decision).
- New finding recorded, not smoothed: uti_dafm_r coverage 92.3% (n=129) ->
  64.3% (n=139), flagged for mentor review.
</commit_message>
<xml_diff>
--- a/experimenting_ml/reports/PROVEN_6_Trust_Report.xlsx
+++ b/experimenting_ml/reports/PROVEN_6_Trust_Report.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,6 +113,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -660,6 +663,13 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Refreshed 6-Sep-2026 against the current, grown dataset (spec.md §9/§18) -- coverage numbers above are LIVE (recomputed via recalibration_check.py's validated methodology), not the original 1-Sep snapshot. Growth is uneven per KPI: wt_ob_lb is still exactly 129 rows (no real AnyLogic round has ever populated WT_OB_LB); wt_ob_a_gb_dub is 159 (item 17's 30 rows only, item 15's 10 excluded); the other 4 are the full 169. Only tt_ob_lb's fixed method (bagged_tree_native) no longer looks like the best choice under this evidence -- mapie_cv_plus is now closer to the 90% target (91.2% vs 85.3%). Flagged for mentor review, NOT changed in code -- see recalibration_check.py / cli_recalibrate_uq_methods.py.</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -743,7 +753,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.962</v>
+        <v>0.853</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>0.9</v>
@@ -772,7 +782,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.923</v>
+        <v>0.912</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>0.9</v>
@@ -801,7 +811,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.962</v>
+        <v>0.875</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>0.9</v>
@@ -830,7 +840,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0.923</v>
+        <v>0.882</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>0.9</v>
@@ -859,7 +869,7 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>0.962</v>
+        <v>0.882</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>0.9</v>
@@ -885,6 +895,13 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>The right-hand "Candidates Flagged"/"Sent to AnyLogic" columns and the full 'Candidate Flagging Decisions' sheet deliberately still reflect round_20260829_181116 exactly as originally exported (28-29 Aug) -- NOT regenerated against the current dataset. That round's 10 candidates are the actual, physical batch still queued for a real AnyLogic Cloud run; re-exporting a fresh batch now would create a second, different candidate set while the first is still pending, and nobody would know which one to actually run. Once round_20260829_181116 is run and ingested, the next export will naturally reflect the grown dataset.</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -893,7 +910,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>Empirical Coverage</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -922,7 +939,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.962</v>
+        <v>0.853</v>
       </c>
       <c r="C21" t="n">
         <v>0.9</v>
@@ -935,7 +952,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.923</v>
+        <v>0.912</v>
       </c>
       <c r="C22" t="n">
         <v>0.9</v>
@@ -948,7 +965,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.962</v>
+        <v>0.875</v>
       </c>
       <c r="C23" t="n">
         <v>0.9</v>
@@ -961,7 +978,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.923</v>
+        <v>0.882</v>
       </c>
       <c r="C24" t="n">
         <v>0.9</v>
@@ -974,7 +991,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.962</v>
+        <v>0.882</v>
       </c>
       <c r="C25" t="n">
         <v>0.9</v>

</xml_diff>